<commit_message>
feat: add team hub, cloud links, and asset download vault
</commit_message>
<xml_diff>
--- a/budget/budget.xlsx
+++ b/budget/budget.xlsx
@@ -505,14 +505,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PRESUPUESTO DE PUESTA EN MARCHA (PILOTO INICIAL) -- PROYECTO EJEMPLO</t>
+          <t>PRESUPUESTO DE PUESTA EN MARCHA (PILOTO INICIAL) -- HIDRO-VIGIA</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Equipo: EQUIPO EJEMPLO | Moneda base: Dolares Estadounidenses (USD) | Metodologia: Costos mayoristas sustentados</t>
+          <t>Equipo: Mentes Pinoleras | Moneda base: Dolares Estadounidenses (USD) | Metodologia: Costos mayoristas sustentados</t>
         </is>
       </c>
     </row>

</xml_diff>